<commit_message>
n8n board refresh 2026-10-08T17:41:58Z
</commit_message>
<xml_diff>
--- a/app/reports/AGMB_research.xlsx
+++ b/app/reports/AGMB_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-07 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-08 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.553</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>8.785</v>
+        <v>8.965</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.553</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.05275000095367432</v>
+        <v>0.05238999843597412</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>49247974.50199203</v>
+        <v>49247978.58337981</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>8.785</v>
+        <v>8.965</v>
       </c>
     </row>
     <row r="38">
@@ -1493,11 +1493,11 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>432643456</v>
+        <v>441508128</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
-        <v>-4.31</v>
+        <v>-4.28</v>
       </c>
       <c r="F5" s="31" t="n"/>
     </row>
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>515196128</v>
+        <v>551259840</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
-        <v>-5.319</v>
+        <v>-4.803</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>55.351</v>
+        <v>49.978</v>
       </c>
     </row>
     <row r="7">
@@ -1535,14 +1535,14 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>873687872</v>
+        <v>893103168</v>
       </c>
       <c r="D7" s="33" t="n"/>
       <c r="E7" s="33" t="n">
-        <v>-1.023</v>
+        <v>-0.974</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>58.275</v>
+        <v>55.476</v>
       </c>
     </row>
     <row r="8">
@@ -1557,14 +1557,14 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>1381160320</v>
+        <v>1389530880</v>
       </c>
       <c r="D8" s="33" t="n"/>
       <c r="E8" s="33" t="n">
-        <v>23.391</v>
+        <v>22.372</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>14.489</v>
+        <v>13.858</v>
       </c>
     </row>
     <row r="9">
@@ -1579,11 +1579,11 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>87186112</v>
+        <v>90673552</v>
       </c>
       <c r="D9" s="33" t="n"/>
       <c r="E9" s="33" t="n">
-        <v>-1.743</v>
+        <v>-1.644</v>
       </c>
       <c r="F9" s="33" t="n"/>
     </row>
@@ -1599,14 +1599,14 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>872262272</v>
+        <v>870580224</v>
       </c>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n">
-        <v>-3.88</v>
+        <v>-3.864</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>5889.007</v>
+        <v>5864.805</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-09T17:41:55Z
</commit_message>
<xml_diff>
--- a/app/reports/AGMB_research.xlsx
+++ b/app/reports/AGMB_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-08 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-09 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.553</v>
+        <v>0.528</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>8.965</v>
+        <v>9.25</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.553</v>
+        <v>0.528</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.05238999843597412</v>
+        <v>0.05245999813079834</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>49247978.58337981</v>
+        <v>49247975.78378379</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>8.965</v>
+        <v>9.25</v>
       </c>
     </row>
     <row r="38">
@@ -1493,11 +1493,11 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>441508128</v>
+        <v>455543776</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
-        <v>-4.28</v>
+        <v>-4.54</v>
       </c>
       <c r="F5" s="31" t="n"/>
     </row>
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>551259840</v>
+        <v>575547712</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
-        <v>-4.803</v>
+        <v>-5.474</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>49.978</v>
+        <v>56.963</v>
       </c>
     </row>
     <row r="7">
@@ -1535,14 +1535,14 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>893103168</v>
+        <v>934522432</v>
       </c>
       <c r="D7" s="33" t="n"/>
       <c r="E7" s="33" t="n">
-        <v>-0.974</v>
+        <v>-1.035</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>55.476</v>
+        <v>58.975</v>
       </c>
     </row>
     <row r="8">
@@ -1557,14 +1557,14 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>1389530880</v>
+        <v>1385345664</v>
       </c>
       <c r="D8" s="33" t="n"/>
       <c r="E8" s="33" t="n">
-        <v>22.372</v>
+        <v>22.627</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>13.858</v>
+        <v>14.016</v>
       </c>
     </row>
     <row r="9">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="D9" s="33" t="n"/>
       <c r="E9" s="33" t="n">
-        <v>-1.644</v>
+        <v>-1.809</v>
       </c>
       <c r="F9" s="33" t="n"/>
     </row>
@@ -1599,14 +1599,14 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>870580224</v>
+        <v>925607232</v>
       </c>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n">
-        <v>-3.864</v>
+        <v>-3.877</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>5864.805</v>
+        <v>5884.166</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-10T17:41:19Z
</commit_message>
<xml_diff>
--- a/app/reports/AGMB_research.xlsx
+++ b/app/reports/AGMB_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-09 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-10 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.528</v>
+        <v>0.543</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>9.25</v>
+        <v>9.08</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.528</v>
+        <v>0.543</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.05245999813079834</v>
+        <v>0.0524399995803833</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>49247975.78378379</v>
+        <v>49247975.33039647</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>9.25</v>
+        <v>9.08</v>
       </c>
     </row>
     <row r="38">
@@ -1493,11 +1493,11 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>455543776</v>
+        <v>447171616</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
-        <v>-4.54</v>
+        <v>-4.46</v>
       </c>
       <c r="F5" s="31" t="n"/>
     </row>
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>575547712</v>
+        <v>563771776</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
-        <v>-5.474</v>
+        <v>-5.543</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>56.963</v>
+        <v>57.679</v>
       </c>
     </row>
     <row r="7">
@@ -1535,14 +1535,14 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>934522432</v>
+        <v>926756288</v>
       </c>
       <c r="D7" s="33" t="n"/>
       <c r="E7" s="33" t="n">
-        <v>-1.035</v>
+        <v>-1.094</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>58.975</v>
+        <v>62.299</v>
       </c>
     </row>
     <row r="8">
@@ -1557,14 +1557,14 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>1385345664</v>
+        <v>1373686528</v>
       </c>
       <c r="D8" s="33" t="n"/>
       <c r="E8" s="33" t="n">
-        <v>22.627</v>
+        <v>22.509</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>14.016</v>
+        <v>13.942</v>
       </c>
     </row>
     <row r="9">
@@ -1579,11 +1579,11 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>90673552</v>
+        <v>89405392</v>
       </c>
       <c r="D9" s="33" t="n"/>
       <c r="E9" s="33" t="n">
-        <v>-1.809</v>
+        <v>-1.71</v>
       </c>
       <c r="F9" s="33" t="n"/>
     </row>
@@ -1599,14 +1599,14 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>925607232</v>
+        <v>913112064</v>
       </c>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n">
-        <v>-3.877</v>
+        <v>-4.157</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>5884.166</v>
+        <v>6310.108</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-12T17:42:29Z
</commit_message>
<xml_diff>
--- a/app/reports/AGMB_research.xlsx
+++ b/app/reports/AGMB_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-11 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-12 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.543</v>
+        <v>0.523</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>9.08</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.543</v>
+        <v>0.523</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.0524399995803833</v>
+        <v>0.05240000247955322</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>49247975.33039647</v>
+        <v>49247975.91397849</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>9.08</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>447171616</v>
+        <v>458006176</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>563771776</v>
+        <v>547579904</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
@@ -1535,7 +1535,7 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>926756288</v>
+        <v>922873280</v>
       </c>
       <c r="D7" s="33" t="n"/>
       <c r="E7" s="33" t="n">
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>1373686528</v>
+        <v>1382505472</v>
       </c>
       <c r="D8" s="33" t="n"/>
       <c r="E8" s="33" t="n">
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>89405392</v>
+        <v>90990592</v>
       </c>
       <c r="D9" s="33" t="n"/>
       <c r="E9" s="33" t="n">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>913112064</v>
+        <v>884036672</v>
       </c>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-13T17:43:01Z
</commit_message>
<xml_diff>
--- a/app/reports/AGMB_research.xlsx
+++ b/app/reports/AGMB_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-12 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-13 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.523</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>8.845000000000001</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.523</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.05240000247955322</v>
+        <v>0.05220999717712402</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>49247975.91397849</v>
+        <v>49247978.2928208</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>9.300000000000001</v>
+        <v>8.845000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>458006176</v>
+        <v>435598368</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>547579904</v>
+        <v>511516160</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
-        <v>-5.543</v>
+        <v>-5.147</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>57.679</v>
+        <v>53.56</v>
       </c>
     </row>
     <row r="7">
@@ -1535,14 +1535,14 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>922873280</v>
+        <v>864627392</v>
       </c>
       <c r="D7" s="33" t="n"/>
       <c r="E7" s="33" t="n">
-        <v>-1.094</v>
+        <v>-1.063</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>62.299</v>
+        <v>60.55</v>
       </c>
     </row>
     <row r="8">
@@ -1557,14 +1557,14 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>1382505472</v>
+        <v>1358738816</v>
       </c>
       <c r="D8" s="33" t="n"/>
       <c r="E8" s="33" t="n">
-        <v>22.509</v>
+        <v>22.55</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>13.942</v>
+        <v>13.968</v>
       </c>
     </row>
     <row r="9">
@@ -1579,11 +1579,11 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>90990592</v>
+        <v>87503152</v>
       </c>
       <c r="D9" s="33" t="n"/>
       <c r="E9" s="33" t="n">
-        <v>-1.71</v>
+        <v>-2.007</v>
       </c>
       <c r="F9" s="33" t="n"/>
     </row>
@@ -1599,14 +1599,14 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>884036672</v>
+        <v>842946624</v>
       </c>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n">
-        <v>-4.157</v>
+        <v>-3.921</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>6310.108</v>
+        <v>5951.93</v>
       </c>
     </row>
     <row r="12">

</xml_diff>